<commit_message>
feat: add Objetivos, Mercado, Conclusoes sheets to Excel workbook
Add three new worksheets to the Excel workbook builder:
- Objetivos: Lists project goals and objectives
- Mercado: Details market segments with descriptions and justifications
- Conclusoes: Summarizes project conclusions, bottleneck notes, layout notes, and improvement recommendations

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_calculos/demonstrativo_calculos.xlsx
+++ b/02_calculos/demonstrativo_calculos.xlsx
@@ -2,18 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="1" r:id="R344d29e04e304d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integrantes" sheetId="2" r:id="R68e028335c264cb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="3" r:id="R66d64bd7281b4cc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Pesquisa" sheetId="4" r:id="R7dd3e5e8659141a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela1_BOM" sheetId="5" r:id="R57ea791720564b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela2_Processos" sheetId="6" r:id="R4c9ae928d1824b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela3_Equipamentos" sheetId="7" r:id="R3cb71a9cb3cd4a9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materiais" sheetId="8" r:id="Raebdf06259fa4bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacidade" sheetId="9" r:id="R1b38a520b92a49e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculo_Router" sheetId="10" r:id="R14b3684dc4e14265"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Areas_Layout" sheetId="11" r:id="Rbfda42ce32034b37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="12" r:id="R00c6119bf078455c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="1" r:id="R85135e82b7a74bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integrantes" sheetId="2" r:id="R669c0b02513a44c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="3" r:id="R6688d53a6ecc445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Pesquisa" sheetId="4" r:id="Ree48396e90a148b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela1_BOM" sheetId="5" r:id="R036f0252e8964561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela2_Processos" sheetId="6" r:id="R97adaee7007b4d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela3_Equipamentos" sheetId="7" r:id="R7c24740dd3214c3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materiais" sheetId="8" r:id="Rabb9174219064177"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacidade" sheetId="9" r:id="R42a76359ac354209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculo_Router" sheetId="10" r:id="Rab6205d5c34d4122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Areas_Layout" sheetId="11" r:id="R59878ec52e6b4a31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="12" r:id="Rdf13f9b4207d4e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivos" sheetId="13" r:id="R5909b206a2b54703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercado" sheetId="14" r:id="R22c8e71cdf914837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conclusoes" sheetId="15" r:id="Rec91dd9ca45f4553"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,18 +35,18 @@
     <x:font>
       <x:b/>
       <x:sz val="14"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="10"/>
-      <x:color rgb="17212B"/>
+      <x:color rgb="FF17212B"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="17212B"/>
+      <x:color rgb="FF17212B"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -56,12 +59,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="17212B"/>
+        <x:fgColor rgb="FF17212B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="E7EEF7"/>
+        <x:fgColor rgb="FFE7EEF7"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -69,30 +72,30 @@
     <x:border/>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="D1D5DB"/>
+        <x:color rgb="FFD1D5DB"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="D1D5DB"/>
+        <x:color rgb="FFD1D5DB"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="D1D5DB"/>
+        <x:color rgb="FFD1D5DB"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="D1D5DB"/>
+        <x:color rgb="FFD1D5DB"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="E5E7EB"/>
+        <x:color rgb="FFE5E7EB"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="E5E7EB"/>
+        <x:color rgb="FFE5E7EB"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="E5E7EB"/>
+        <x:color rgb="FFE5E7EB"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="E5E7EB"/>
+        <x:color rgb="FFE5E7EB"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -960,6 +963,216 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Objetivos do projeto</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="8" t="str">
+        <x:v>Objetivo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
+        <x:v>Desenvolver proposta básica de fábrica para o Kit para Churrasco Tramontina 3 Peças (ref. 22399036), com meta semanal de 1.000 kits bons.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Dimensionar processos, equipamentos e arranjo físico para integrar setor metálico, setor madeira, montagem e embalagem em fluxo contínuo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Calcular quantidades de equipamentos com base em tempos-padrão estimados, eficiência, confiabilidade e rendimento de processo explicitados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
+        <x:v>Selecionar segmentos de mercado visados e justificar a meta de produção proposta.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="12" t="str">
+        <x:v>Gerar documentação técnica auditável — tabelas, fluxograma, mapofluxograma, layout esquemático e memória de cálculo — com todas as fontes identificadas.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Segmentos de mercado</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="8" t="str">
+        <x:v>Segmento</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>Descrição</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>Justificativa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
+        <x:v>Varejo doméstico de churrasco</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>Supermercados, lojas de utilidades domésticas, redes especializadas em artigos para churrasco e grill.</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>O Brasil possui cultura de churrasco consolidada com consumo frequente em todas as regiões. O produto Tramontina tem reconhecimento nacional de qualidade, garantia de 5 anos e distribuição em redes de varejo de grande porte.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Kits presente e gift sets sazonais</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Embalagem blister/cartela posiciona o produto como presente premium em datas comemorativas.</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Dia dos Pais, Natal e Dia dos Namorados concentram picos de demanda por kits de churrasco. A embalagem compacta (1,23 kg, 38,9 cm de altura) facilita o transporte e o presenteamento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>E-commerce e marketplaces</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>Venda direta em plataformas como Mercado Livre, Amazon Brasil, Shopee e site próprio Tramontina.</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>As dimensões compactas da embalagem (38,9 × 4,0 × 21,6 cm, 1,23 kg) são favoráveis ao custo de frete e compatíveis com restrições de tamanho das plataformas. O produto já está disponível no e-commerce oficial da Tramontina.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
+        <x:v>Brindes corporativos e programas de fidelidade</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>Empresas que oferecem brindes premium para clientes, colaboradores e ações de marketing.</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>A certificação FSC C125626 da madeira e a marca Tramontina reforçam o apelo sustentável, relevante para empresas com compromissos ESG. O kit representa um brinde de alto valor percebido com custo unitário moderado.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Conclusoes do projeto</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="8" t="str">
+        <x:v>Tópico</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>Conteúdo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
+        <x:v>Resumo</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>O projeto propõe uma fábrica de 384 m² (24 m × 16 m) capaz de produzir 1.000 kits bons/semana (demanda bruta calculada de 1.053 kits/semana) em regime de 1 turno de 7 h úteis/dia, 5 dias/semana. A ocupação do espaço é de 67,8%, com área requerida estimada de 260,4 m².</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Gargalo</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>O gargalo identificado é o Router CNC (Maksiwa RTC.1313), com utilização de 65,4% para 2 unidades. A operação de fresagem do sulco da tábua e usinagem dos cabos tem o maior tempo-padrão estimado (120 s/kit). Para dobrar a capacidade sem alterar o prédio, seria necessário adicionar um terceiro turno ou uma terceira unidade do Router CNC.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Layout</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>O arranjo físico proposto é misto: setores funcionais para metal e madeira (com equipamentos agrupados por processo) e fluxo em célula/linha para montagem e embalagem. A folga de 32,2% da área (123,6 m²) permite expansão futura sem reforma estrutural.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
+        <x:v>Melhoria 1</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>Realizar estudo de tempos real (cronoanálise) no chão de fábrica para substituir os tempos-padrão estimados por valores medidos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="12" t="str">
+        <x:v>Melhoria 2</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>Cotar equipamentos com pelo menos dois fornecedores alternativos para validar capacidades e dimensões antes de fechar o layout definitivo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="12" t="str">
+        <x:v>Melhoria 3</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>Conduzir um piloto de produção de 1 semana para validar o rendimento final de 95% e as taxas de eficiência e confiabilidade assumidas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="str">
+        <x:v>Melhoria 4</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>Avaliar implantação de Controle Estatístico de Processo (CEP) nas etapas críticas de tratamento térmico e afiação para reduzir variabilidade de qualidade.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="str">
+        <x:v>Melhoria 5</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="str">
+        <x:v>Modelar cenários de demanda (±30%) para dimensionar plano de capacidade de resposta sem ociosidade excessiva ou gargalos adicionais.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="str">
+        <x:v>Melhoria 6</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>Incluir análise de custo de implantação e payback como complemento ao projeto básico de fábrica.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
fix: mapofluxograma — inline QC nodes, grid-pattern routing, elbow edges for zone crossings
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_calculos/demonstrativo_calculos.xlsx
+++ b/02_calculos/demonstrativo_calculos.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="1" r:id="R85135e82b7a74bfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integrantes" sheetId="2" r:id="R669c0b02513a44c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="3" r:id="R6688d53a6ecc445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Pesquisa" sheetId="4" r:id="Ree48396e90a148b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela1_BOM" sheetId="5" r:id="R036f0252e8964561"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela2_Processos" sheetId="6" r:id="R97adaee7007b4d9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela3_Equipamentos" sheetId="7" r:id="R7c24740dd3214c3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materiais" sheetId="8" r:id="Rabb9174219064177"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacidade" sheetId="9" r:id="R42a76359ac354209"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculo_Router" sheetId="10" r:id="Rab6205d5c34d4122"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Areas_Layout" sheetId="11" r:id="R59878ec52e6b4a31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="12" r:id="Rdf13f9b4207d4e05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivos" sheetId="13" r:id="R5909b206a2b54703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercado" sheetId="14" r:id="R22c8e71cdf914837"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conclusoes" sheetId="15" r:id="Rec91dd9ca45f4553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="1" r:id="Rd361690e2b084108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integrantes" sheetId="2" r:id="Ra4a63c51586f41ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="3" r:id="R7bbf9ce1bec94208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Pesquisa" sheetId="4" r:id="R14765efbb31e4fb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela1_BOM" sheetId="5" r:id="R8e5df6b9e4e54366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela2_Processos" sheetId="6" r:id="Rb9a7aba956744f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela3_Equipamentos" sheetId="7" r:id="R7bacc32c74f94fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materiais" sheetId="8" r:id="R82d6bc213a794530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacidade" sheetId="9" r:id="Ree245b6c2a094389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculo_Router" sheetId="10" r:id="R0f492d77fe2144a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Areas_Layout" sheetId="11" r:id="R5a8e9c41f37d491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="12" r:id="Rd2d74c8d3ab74b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivos" sheetId="13" r:id="Rcbeb535080e44c49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercado" sheetId="14" r:id="Rc449521c5769448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conclusoes" sheetId="15" r:id="Ra7b97f0acb3347ad"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>